<commit_message>
LCSC Links ko Custom Supplier kr dia ha or price bardha di ha
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Digikey_BOM.xlsx
+++ b/Deliverables/BOM/Digikey_BOM.xlsx
@@ -12,7 +12,7 @@
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
   </bookViews>
   <sheets>
-    <sheet name="Refrence " sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913" concurrentCalc="0"/>
   <extLst>
@@ -176,9 +176,6 @@
     <t>Link</t>
   </si>
   <si>
-    <t xml:space="preserve">Bill of Material (BOM) for Refrence Formate </t>
-  </si>
-  <si>
     <t>CAP CER 10UF 35V X5R 0603</t>
   </si>
   <si>
@@ -602,9 +599,6 @@
     <t xml:space="preserve">Seiko </t>
   </si>
   <si>
-    <t>LCSC</t>
-  </si>
-  <si>
     <t xml:space="preserve">SMD2012-2P Crystals ROHS
 </t>
   </si>
@@ -651,6 +645,12 @@
   </si>
   <si>
     <t xml:space="preserve">Alternate Part use Footprint need to be change in design </t>
+  </si>
+  <si>
+    <t>Custom supplier</t>
+  </si>
+  <si>
+    <t>Bill of Material (BOM) for Saleem Custom Product</t>
   </si>
 </sst>
 </file>
@@ -1157,6 +1157,206 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1168,206 +1368,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1664,7 +1664,7 @@
     <col min="9" max="9" width="11.28515625" style="10" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19.42578125" style="10" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="18.7109375" bestFit="1" customWidth="1"/>
@@ -1673,25 +1673,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="22"/>
+      <c r="A1" s="88" t="s">
+        <v>205</v>
+      </c>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="89"/>
+      <c r="O1" s="89"/>
+      <c r="P1" s="89"/>
+      <c r="Q1" s="90"/>
     </row>
     <row r="2" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -1750,55 +1750,55 @@
       <c r="A3" s="13">
         <v>1</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="83" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="64" t="s">
+      <c r="C3" s="56" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="57" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="65" t="s">
+      <c r="E3" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="E3" s="38" t="s">
+      <c r="F3" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="F3" s="38" t="s">
-        <v>54</v>
-      </c>
-      <c r="G3" s="23" t="s">
-        <v>167</v>
-      </c>
-      <c r="H3" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="I3" s="38" t="s">
+      <c r="G3" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="I3" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="J3" s="45">
+      <c r="J3" s="38">
         <v>1</v>
       </c>
-      <c r="K3" s="25">
+      <c r="K3" s="21">
         <f>J3*5</f>
         <v>5</v>
       </c>
-      <c r="L3" s="66" t="s">
+      <c r="L3" s="58" t="s">
         <v>30</v>
       </c>
-      <c r="M3" s="27">
+      <c r="M3" s="23">
         <v>0.45</v>
       </c>
-      <c r="N3" s="27">
+      <c r="N3" s="23">
         <f>M3*J3</f>
         <v>0.45</v>
       </c>
-      <c r="O3" s="27">
+      <c r="O3" s="23">
         <v>0.45</v>
       </c>
-      <c r="P3" s="27">
+      <c r="P3" s="23">
         <f>O3*K3</f>
         <v>2.25</v>
       </c>
-      <c r="Q3" s="28"/>
+      <c r="Q3" s="24"/>
       <c r="R3" s="2"/>
       <c r="S3" s="2"/>
     </row>
@@ -1806,24 +1806,24 @@
       <c r="A4" s="13">
         <v>2</v>
       </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="67" t="s">
+      <c r="B4" s="84"/>
+      <c r="C4" s="59" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="60" t="s">
         <v>55</v>
       </c>
-      <c r="D4" s="68" t="s">
+      <c r="E4" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="F4" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F4" s="14" t="s">
-        <v>58</v>
-      </c>
       <c r="G4" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I4" s="14" t="s">
         <v>6</v>
@@ -1852,7 +1852,7 @@
         <f t="shared" ref="P4:P39" si="2">O4*K4</f>
         <v>5.6499999999999995</v>
       </c>
-      <c r="Q4" s="29"/>
+      <c r="Q4" s="25"/>
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
     </row>
@@ -1860,27 +1860,27 @@
       <c r="A5" s="13">
         <v>3</v>
       </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="67" t="s">
+      <c r="B5" s="84"/>
+      <c r="C5" s="59" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="60" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="68" t="s">
+      <c r="E5" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="E5" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>61</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J5" s="12">
         <v>1</v>
@@ -1906,7 +1906,7 @@
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q5" s="29"/>
+      <c r="Q5" s="25"/>
       <c r="R5" s="2"/>
       <c r="S5" s="2"/>
     </row>
@@ -1914,27 +1914,27 @@
       <c r="A6" s="13">
         <v>4</v>
       </c>
-      <c r="B6" s="36"/>
-      <c r="C6" s="67" t="s">
+      <c r="B6" s="84"/>
+      <c r="C6" s="59" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" s="60" t="s">
         <v>62</v>
       </c>
-      <c r="D6" s="68" t="s">
+      <c r="E6" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>64</v>
-      </c>
       <c r="G6" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J6" s="12">
         <v>2</v>
@@ -1960,7 +1960,7 @@
         <f t="shared" si="2"/>
         <v>0.37</v>
       </c>
-      <c r="Q6" s="29"/>
+      <c r="Q6" s="25"/>
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
     </row>
@@ -1968,24 +1968,24 @@
       <c r="A7" s="13">
         <v>5</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="67" t="s">
+      <c r="B7" s="84"/>
+      <c r="C7" s="59" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="60" t="s">
         <v>65</v>
       </c>
-      <c r="D7" s="68" t="s">
+      <c r="E7" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="E7" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>67</v>
-      </c>
       <c r="G7" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I7" s="14" t="s">
         <v>4</v>
@@ -2014,7 +2014,7 @@
         <f t="shared" si="2"/>
         <v>5.3759999999999994</v>
       </c>
-      <c r="Q7" s="29"/>
+      <c r="Q7" s="25"/>
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
     </row>
@@ -2022,24 +2022,24 @@
       <c r="A8" s="13">
         <v>6</v>
       </c>
-      <c r="B8" s="36"/>
-      <c r="C8" s="67" t="s">
+      <c r="B8" s="84"/>
+      <c r="C8" s="59" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" s="60" t="s">
         <v>68</v>
-      </c>
-      <c r="D8" s="68" t="s">
-        <v>69</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="F8" s="69" t="s">
-        <v>70</v>
+      <c r="F8" s="61" t="s">
+        <v>69</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="I8" s="14" t="s">
         <v>35</v>
@@ -2068,8 +2068,8 @@
         <f t="shared" si="2"/>
         <v>4.3</v>
       </c>
-      <c r="Q8" s="86" t="s">
-        <v>205</v>
+      <c r="Q8" s="78" t="s">
+        <v>203</v>
       </c>
       <c r="R8" s="2"/>
       <c r="S8" s="2"/>
@@ -2078,24 +2078,24 @@
       <c r="A9" s="13">
         <v>7</v>
       </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="70" t="s">
+      <c r="B9" s="84"/>
+      <c r="C9" s="62" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" s="63" t="s">
         <v>71</v>
       </c>
-      <c r="D9" s="71" t="s">
+      <c r="E9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>73</v>
-      </c>
       <c r="G9" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I9" s="14" t="s">
         <v>34</v>
@@ -2124,7 +2124,7 @@
         <f t="shared" si="2"/>
         <v>2.9400000000000004</v>
       </c>
-      <c r="Q9" s="29"/>
+      <c r="Q9" s="25"/>
       <c r="R9" s="2"/>
       <c r="S9" s="2"/>
     </row>
@@ -2132,24 +2132,24 @@
       <c r="A10" s="13">
         <v>8</v>
       </c>
-      <c r="B10" s="36"/>
-      <c r="C10" s="67" t="s">
+      <c r="B10" s="84"/>
+      <c r="C10" s="59" t="s">
+        <v>73</v>
+      </c>
+      <c r="D10" s="60" t="s">
         <v>74</v>
       </c>
-      <c r="D10" s="68" t="s">
+      <c r="E10" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" s="14" t="s">
         <v>75</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>76</v>
       </c>
       <c r="G10" s="16" t="s">
         <v>5</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I10" s="14" t="s">
         <v>7</v>
@@ -2178,7 +2178,7 @@
         <f t="shared" si="2"/>
         <v>2.5</v>
       </c>
-      <c r="Q10" s="29"/>
+      <c r="Q10" s="25"/>
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
     </row>
@@ -2186,27 +2186,27 @@
       <c r="A11" s="13">
         <v>9</v>
       </c>
-      <c r="B11" s="36"/>
-      <c r="C11" s="67" t="s">
+      <c r="B11" s="84"/>
+      <c r="C11" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="60" t="s">
         <v>77</v>
       </c>
-      <c r="D11" s="68" t="s">
+      <c r="E11" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="E11" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>79</v>
-      </c>
       <c r="G11" s="16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J11" s="12">
         <v>2</v>
@@ -2232,7 +2232,7 @@
         <f t="shared" si="2"/>
         <v>0.48</v>
       </c>
-      <c r="Q11" s="29"/>
+      <c r="Q11" s="25"/>
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
     </row>
@@ -2240,53 +2240,53 @@
       <c r="A12" s="13">
         <v>10</v>
       </c>
-      <c r="B12" s="37"/>
-      <c r="C12" s="72" t="s">
+      <c r="B12" s="85"/>
+      <c r="C12" s="64" t="s">
+        <v>79</v>
+      </c>
+      <c r="D12" s="65" t="s">
         <v>80</v>
       </c>
-      <c r="D12" s="73" t="s">
+      <c r="E12" s="66" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="66" t="s">
         <v>81</v>
       </c>
-      <c r="E12" s="74" t="s">
-        <v>53</v>
-      </c>
-      <c r="F12" s="74" t="s">
-        <v>82</v>
-      </c>
-      <c r="G12" s="30" t="s">
-        <v>171</v>
-      </c>
-      <c r="H12" s="31" t="s">
-        <v>128</v>
-      </c>
-      <c r="I12" s="74" t="s">
-        <v>86</v>
-      </c>
-      <c r="J12" s="46">
+      <c r="G12" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="H12" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="I12" s="66" t="s">
+        <v>85</v>
+      </c>
+      <c r="J12" s="39">
         <v>2</v>
       </c>
-      <c r="K12" s="32">
+      <c r="K12" s="28">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L12" s="75" t="s">
+      <c r="L12" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="M12" s="33">
+      <c r="M12" s="29">
         <v>0.1</v>
       </c>
-      <c r="N12" s="33">
+      <c r="N12" s="29">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
-      <c r="O12" s="33">
+      <c r="O12" s="29">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="P12" s="33">
+      <c r="P12" s="29">
         <f t="shared" si="2"/>
         <v>0.49</v>
       </c>
-      <c r="Q12" s="34"/>
+      <c r="Q12" s="30"/>
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
     </row>
@@ -2294,55 +2294,55 @@
       <c r="A13" s="13">
         <v>11</v>
       </c>
-      <c r="B13" s="35" t="s">
+      <c r="B13" s="83" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="64" t="s">
+      <c r="C13" s="56" t="s">
+        <v>86</v>
+      </c>
+      <c r="D13" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="D13" s="65" t="s">
+      <c r="E13" s="31" t="s">
+        <v>164</v>
+      </c>
+      <c r="F13" s="31" t="s">
         <v>88</v>
       </c>
-      <c r="E13" s="38" t="s">
-        <v>165</v>
-      </c>
-      <c r="F13" s="38" t="s">
-        <v>89</v>
-      </c>
-      <c r="G13" s="23" t="s">
-        <v>172</v>
-      </c>
-      <c r="H13" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="I13" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="J13" s="45">
+      <c r="G13" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="H13" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="I13" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="J13" s="38">
         <v>4</v>
       </c>
-      <c r="K13" s="25">
+      <c r="K13" s="21">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="L13" s="66" t="s">
+      <c r="L13" s="58" t="s">
         <v>30</v>
       </c>
-      <c r="M13" s="27">
+      <c r="M13" s="23">
         <v>0.25</v>
       </c>
-      <c r="N13" s="27">
+      <c r="N13" s="23">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="O13" s="27">
+      <c r="O13" s="23">
         <v>0.20499999999999999</v>
       </c>
-      <c r="P13" s="27">
+      <c r="P13" s="23">
         <f t="shared" si="2"/>
         <v>4.0999999999999996</v>
       </c>
-      <c r="Q13" s="44"/>
+      <c r="Q13" s="37"/>
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
     </row>
@@ -2350,53 +2350,53 @@
       <c r="A14" s="13">
         <v>12</v>
       </c>
-      <c r="B14" s="37"/>
-      <c r="C14" s="76" t="s">
-        <v>196</v>
-      </c>
-      <c r="D14" s="73" t="s">
+      <c r="B14" s="85"/>
+      <c r="C14" s="68" t="s">
+        <v>194</v>
+      </c>
+      <c r="D14" s="65" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="74" t="s">
-        <v>166</v>
-      </c>
-      <c r="F14" s="74" t="s">
-        <v>90</v>
-      </c>
-      <c r="G14" s="30" t="s">
-        <v>173</v>
-      </c>
-      <c r="H14" s="31" t="s">
-        <v>128</v>
-      </c>
-      <c r="I14" s="30" t="s">
-        <v>128</v>
-      </c>
-      <c r="J14" s="46">
+      <c r="E14" s="66" t="s">
+        <v>165</v>
+      </c>
+      <c r="F14" s="66" t="s">
+        <v>89</v>
+      </c>
+      <c r="G14" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="H14" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="I14" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="J14" s="39">
         <v>2</v>
       </c>
-      <c r="K14" s="32">
+      <c r="K14" s="28">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L14" s="75" t="s">
+      <c r="L14" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="M14" s="33">
+      <c r="M14" s="29">
         <v>0.97</v>
       </c>
-      <c r="N14" s="33">
+      <c r="N14" s="29">
         <f t="shared" si="1"/>
         <v>1.94</v>
       </c>
-      <c r="O14" s="33">
+      <c r="O14" s="29">
         <v>0.86399999999999999</v>
       </c>
-      <c r="P14" s="33">
+      <c r="P14" s="29">
         <f t="shared" si="2"/>
         <v>8.64</v>
       </c>
-      <c r="Q14" s="34"/>
+      <c r="Q14" s="30"/>
       <c r="R14" s="2"/>
       <c r="S14" s="2"/>
     </row>
@@ -2404,55 +2404,55 @@
       <c r="A15" s="13">
         <v>13</v>
       </c>
-      <c r="B15" s="43" t="s">
+      <c r="B15" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="77" t="s">
+      <c r="C15" s="69" t="s">
+        <v>90</v>
+      </c>
+      <c r="D15" s="70" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="71" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" s="71" t="s">
         <v>91</v>
       </c>
-      <c r="D15" s="78" t="s">
-        <v>40</v>
-      </c>
-      <c r="E15" s="79" t="s">
-        <v>31</v>
-      </c>
-      <c r="F15" s="79" t="s">
-        <v>92</v>
-      </c>
-      <c r="G15" s="47" t="s">
-        <v>174</v>
-      </c>
-      <c r="H15" s="48" t="s">
-        <v>128</v>
-      </c>
-      <c r="I15" s="79" t="s">
-        <v>96</v>
-      </c>
-      <c r="J15" s="49">
+      <c r="G15" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="H15" s="41" t="s">
+        <v>127</v>
+      </c>
+      <c r="I15" s="71" t="s">
+        <v>95</v>
+      </c>
+      <c r="J15" s="42">
         <v>1</v>
       </c>
-      <c r="K15" s="50">
+      <c r="K15" s="43">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L15" s="80" t="s">
+      <c r="L15" s="72" t="s">
         <v>30</v>
       </c>
-      <c r="M15" s="51">
+      <c r="M15" s="44">
         <v>0.92</v>
       </c>
-      <c r="N15" s="51">
+      <c r="N15" s="44">
         <f t="shared" si="1"/>
         <v>0.92</v>
       </c>
-      <c r="O15" s="51">
+      <c r="O15" s="44">
         <v>0.92</v>
       </c>
-      <c r="P15" s="51">
+      <c r="P15" s="44">
         <f t="shared" si="2"/>
         <v>4.6000000000000005</v>
       </c>
-      <c r="Q15" s="62"/>
+      <c r="Q15" s="54"/>
       <c r="R15" s="2"/>
       <c r="S15" s="2"/>
     </row>
@@ -2460,55 +2460,55 @@
       <c r="A16" s="13">
         <v>14</v>
       </c>
-      <c r="B16" s="52" t="s">
+      <c r="B16" s="45" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="81" t="s">
+      <c r="C16" s="73" t="s">
+        <v>92</v>
+      </c>
+      <c r="D16" s="74" t="s">
         <v>93</v>
       </c>
-      <c r="D16" s="82" t="s">
+      <c r="E16" s="46" t="s">
+        <v>45</v>
+      </c>
+      <c r="F16" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="E16" s="53" t="s">
-        <v>45</v>
-      </c>
-      <c r="F16" s="53" t="s">
-        <v>95</v>
-      </c>
-      <c r="G16" s="53" t="s">
-        <v>175</v>
-      </c>
-      <c r="H16" s="54" t="s">
-        <v>128</v>
-      </c>
-      <c r="I16" s="53" t="s">
-        <v>128</v>
-      </c>
-      <c r="J16" s="55">
+      <c r="G16" s="46" t="s">
+        <v>174</v>
+      </c>
+      <c r="H16" s="47" t="s">
+        <v>127</v>
+      </c>
+      <c r="I16" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="J16" s="48">
         <v>1</v>
       </c>
-      <c r="K16" s="56">
+      <c r="K16" s="49">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L16" s="83" t="s">
+      <c r="L16" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="M16" s="57">
+      <c r="M16" s="50">
         <v>0.14000000000000001</v>
       </c>
-      <c r="N16" s="58">
+      <c r="N16" s="51">
         <f t="shared" si="1"/>
         <v>0.14000000000000001</v>
       </c>
-      <c r="O16" s="58">
+      <c r="O16" s="51">
         <v>0.14000000000000001</v>
       </c>
-      <c r="P16" s="58">
+      <c r="P16" s="51">
         <f t="shared" si="2"/>
         <v>0.70000000000000007</v>
       </c>
-      <c r="Q16" s="59"/>
+      <c r="Q16" s="52"/>
       <c r="R16" s="2"/>
       <c r="S16" s="2"/>
     </row>
@@ -2516,55 +2516,55 @@
       <c r="A17" s="13">
         <v>15</v>
       </c>
-      <c r="B17" s="35" t="s">
+      <c r="B17" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="64" t="s">
+      <c r="C17" s="56" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" s="57" t="s">
         <v>97</v>
       </c>
-      <c r="D17" s="65" t="s">
+      <c r="E17" s="31" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="31" t="s">
         <v>98</v>
       </c>
-      <c r="E17" s="38" t="s">
-        <v>46</v>
-      </c>
-      <c r="F17" s="38" t="s">
-        <v>99</v>
-      </c>
-      <c r="G17" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="H17" s="39" t="s">
-        <v>128</v>
-      </c>
-      <c r="I17" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="J17" s="45">
+      <c r="G17" s="31" t="s">
+        <v>175</v>
+      </c>
+      <c r="H17" s="32" t="s">
+        <v>127</v>
+      </c>
+      <c r="I17" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="J17" s="38">
         <v>1</v>
       </c>
-      <c r="K17" s="25">
+      <c r="K17" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L17" s="66" t="s">
+      <c r="L17" s="58" t="s">
         <v>30</v>
       </c>
-      <c r="M17" s="40">
+      <c r="M17" s="33">
         <v>0.1</v>
       </c>
-      <c r="N17" s="27">
+      <c r="N17" s="23">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="O17" s="27">
+      <c r="O17" s="23">
         <v>0.1</v>
       </c>
-      <c r="P17" s="27">
+      <c r="P17" s="23">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q17" s="41"/>
+      <c r="Q17" s="34"/>
       <c r="R17" s="2"/>
       <c r="S17" s="2"/>
     </row>
@@ -2572,24 +2572,24 @@
       <c r="A18" s="13">
         <v>16</v>
       </c>
-      <c r="B18" s="36"/>
-      <c r="C18" s="67" t="s">
+      <c r="B18" s="84"/>
+      <c r="C18" s="59" t="s">
+        <v>99</v>
+      </c>
+      <c r="D18" s="60" t="s">
         <v>100</v>
-      </c>
-      <c r="D18" s="68" t="s">
-        <v>101</v>
       </c>
       <c r="E18" s="14" t="s">
         <v>46</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I18" s="14" t="s">
         <v>12</v>
@@ -2618,7 +2618,7 @@
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q18" s="42"/>
+      <c r="Q18" s="35"/>
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
     </row>
@@ -2626,27 +2626,27 @@
       <c r="A19" s="13">
         <v>17</v>
       </c>
-      <c r="B19" s="36"/>
-      <c r="C19" s="67" t="s">
-        <v>103</v>
-      </c>
-      <c r="D19" s="68" t="s">
+      <c r="B19" s="84"/>
+      <c r="C19" s="59" t="s">
+        <v>102</v>
+      </c>
+      <c r="D19" s="60" t="s">
         <v>37</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>46</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J19" s="12">
         <v>1</v>
@@ -2672,7 +2672,7 @@
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q19" s="42"/>
+      <c r="Q19" s="35"/>
       <c r="R19" s="2"/>
       <c r="S19" s="2"/>
     </row>
@@ -2680,24 +2680,24 @@
       <c r="A20" s="13">
         <v>18</v>
       </c>
-      <c r="B20" s="36"/>
-      <c r="C20" s="67" t="s">
+      <c r="B20" s="84"/>
+      <c r="C20" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" s="60" t="s">
         <v>105</v>
-      </c>
-      <c r="D20" s="68" t="s">
-        <v>106</v>
       </c>
       <c r="E20" s="14" t="s">
         <v>46</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I20" s="14" t="s">
         <v>38</v>
@@ -2726,7 +2726,7 @@
         <f t="shared" si="2"/>
         <v>0.72</v>
       </c>
-      <c r="Q20" s="29"/>
+      <c r="Q20" s="25"/>
       <c r="R20" s="2"/>
       <c r="S20" s="2"/>
     </row>
@@ -2734,27 +2734,27 @@
       <c r="A21" s="13">
         <v>19</v>
       </c>
-      <c r="B21" s="36"/>
-      <c r="C21" s="70" t="s">
+      <c r="B21" s="84"/>
+      <c r="C21" s="62" t="s">
+        <v>195</v>
+      </c>
+      <c r="D21" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="F21" s="14" t="s">
         <v>197</v>
       </c>
-      <c r="D21" s="68" t="s">
-        <v>108</v>
-      </c>
-      <c r="E21" s="14" t="s">
+      <c r="G21" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="F21" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>200</v>
-      </c>
       <c r="H21" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J21" s="12">
         <v>4</v>
@@ -2780,7 +2780,7 @@
         <f t="shared" si="2"/>
         <v>5.0600000000000005</v>
       </c>
-      <c r="Q21" s="29"/>
+      <c r="Q21" s="25"/>
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
     </row>
@@ -2788,27 +2788,27 @@
       <c r="A22" s="13">
         <v>20</v>
       </c>
-      <c r="B22" s="36"/>
-      <c r="C22" s="67" t="s">
+      <c r="B22" s="84"/>
+      <c r="C22" s="59" t="s">
+        <v>108</v>
+      </c>
+      <c r="D22" s="60" t="s">
         <v>109</v>
-      </c>
-      <c r="D22" s="68" t="s">
-        <v>110</v>
       </c>
       <c r="E22" s="14" t="s">
         <v>46</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J22" s="12">
         <v>4</v>
@@ -2834,7 +2834,7 @@
         <f t="shared" si="2"/>
         <v>0.48</v>
       </c>
-      <c r="Q22" s="29"/>
+      <c r="Q22" s="25"/>
       <c r="R22" s="2"/>
       <c r="S22" s="2"/>
     </row>
@@ -2842,27 +2842,27 @@
       <c r="A23" s="13">
         <v>21</v>
       </c>
-      <c r="B23" s="36"/>
-      <c r="C23" s="67" t="s">
+      <c r="B23" s="84"/>
+      <c r="C23" s="59" t="s">
+        <v>111</v>
+      </c>
+      <c r="D23" s="60" t="s">
         <v>112</v>
-      </c>
-      <c r="D23" s="68" t="s">
-        <v>113</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>46</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J23" s="12">
         <v>4</v>
@@ -2888,7 +2888,7 @@
         <f t="shared" si="2"/>
         <v>3.02</v>
       </c>
-      <c r="Q23" s="29"/>
+      <c r="Q23" s="25"/>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
     </row>
@@ -2896,27 +2896,27 @@
       <c r="A24" s="13">
         <v>22</v>
       </c>
-      <c r="B24" s="36"/>
-      <c r="C24" s="67" t="s">
+      <c r="B24" s="84"/>
+      <c r="C24" s="59" t="s">
+        <v>114</v>
+      </c>
+      <c r="D24" s="60" t="s">
         <v>115</v>
-      </c>
-      <c r="D24" s="68" t="s">
-        <v>116</v>
       </c>
       <c r="E24" s="14" t="s">
         <v>46</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J24" s="12">
         <v>1</v>
@@ -2942,7 +2942,7 @@
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q24" s="29"/>
+      <c r="Q24" s="25"/>
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
     </row>
@@ -2950,53 +2950,53 @@
       <c r="A25" s="13">
         <v>23</v>
       </c>
-      <c r="B25" s="37"/>
-      <c r="C25" s="72" t="s">
+      <c r="B25" s="85"/>
+      <c r="C25" s="64" t="s">
+        <v>117</v>
+      </c>
+      <c r="D25" s="65" t="s">
         <v>118</v>
       </c>
-      <c r="D25" s="73" t="s">
+      <c r="E25" s="66" t="s">
+        <v>46</v>
+      </c>
+      <c r="F25" s="66" t="s">
         <v>119</v>
       </c>
-      <c r="E25" s="74" t="s">
-        <v>46</v>
-      </c>
-      <c r="F25" s="74" t="s">
-        <v>120</v>
-      </c>
-      <c r="G25" s="30" t="s">
-        <v>169</v>
-      </c>
-      <c r="H25" s="30" t="s">
-        <v>128</v>
-      </c>
-      <c r="I25" s="74" t="s">
-        <v>127</v>
-      </c>
-      <c r="J25" s="46">
+      <c r="G25" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="H25" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="I25" s="66" t="s">
+        <v>126</v>
+      </c>
+      <c r="J25" s="39">
         <v>1</v>
       </c>
-      <c r="K25" s="32">
+      <c r="K25" s="28">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L25" s="75" t="s">
+      <c r="L25" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="M25" s="33">
+      <c r="M25" s="29">
         <v>0.1</v>
       </c>
-      <c r="N25" s="33">
+      <c r="N25" s="29">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="O25" s="33">
+      <c r="O25" s="29">
         <v>0.1</v>
       </c>
-      <c r="P25" s="33">
+      <c r="P25" s="29">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q25" s="34"/>
+      <c r="Q25" s="30"/>
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
     </row>
@@ -3004,55 +3004,55 @@
       <c r="A26" s="13">
         <v>24</v>
       </c>
-      <c r="B26" s="35" t="s">
-        <v>140</v>
-      </c>
-      <c r="C26" s="64" t="s">
+      <c r="B26" s="83" t="s">
+        <v>139</v>
+      </c>
+      <c r="C26" s="56" t="s">
+        <v>128</v>
+      </c>
+      <c r="D26" s="57" t="s">
         <v>129</v>
       </c>
-      <c r="D26" s="65" t="s">
+      <c r="E26" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="F26" s="31" t="s">
         <v>130</v>
       </c>
-      <c r="E26" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="F26" s="38" t="s">
-        <v>131</v>
-      </c>
-      <c r="G26" s="23" t="s">
-        <v>178</v>
-      </c>
-      <c r="H26" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="I26" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="J26" s="45">
+      <c r="G26" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="H26" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="I26" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="J26" s="38">
         <v>2</v>
       </c>
-      <c r="K26" s="25">
+      <c r="K26" s="21">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L26" s="66" t="s">
+      <c r="L26" s="58" t="s">
         <v>30</v>
       </c>
-      <c r="M26" s="27">
+      <c r="M26" s="23">
         <v>0.96</v>
       </c>
-      <c r="N26" s="27">
+      <c r="N26" s="23">
         <f t="shared" si="1"/>
         <v>1.92</v>
       </c>
-      <c r="O26" s="27">
+      <c r="O26" s="23">
         <v>0.96</v>
       </c>
-      <c r="P26" s="27">
+      <c r="P26" s="23">
         <f t="shared" si="2"/>
         <v>9.6</v>
       </c>
-      <c r="Q26" s="28"/>
+      <c r="Q26" s="24"/>
       <c r="R26" s="2"/>
       <c r="S26" s="2"/>
     </row>
@@ -3060,53 +3060,53 @@
       <c r="A27" s="13">
         <v>25</v>
       </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="87" t="s">
+      <c r="B27" s="85"/>
+      <c r="C27" s="79" t="s">
+        <v>131</v>
+      </c>
+      <c r="D27" s="80" t="s">
         <v>132</v>
       </c>
-      <c r="D27" s="88" t="s">
+      <c r="E27" s="80" t="s">
+        <v>31</v>
+      </c>
+      <c r="F27" s="80" t="s">
         <v>133</v>
       </c>
-      <c r="E27" s="88" t="s">
-        <v>31</v>
-      </c>
-      <c r="F27" s="88" t="s">
-        <v>134</v>
-      </c>
-      <c r="G27" s="89" t="s">
-        <v>190</v>
-      </c>
-      <c r="H27" s="89" t="s">
-        <v>128</v>
-      </c>
-      <c r="I27" s="89" t="s">
-        <v>128</v>
-      </c>
-      <c r="J27" s="46">
+      <c r="G27" s="81" t="s">
+        <v>189</v>
+      </c>
+      <c r="H27" s="81" t="s">
+        <v>127</v>
+      </c>
+      <c r="I27" s="81" t="s">
+        <v>127</v>
+      </c>
+      <c r="J27" s="39">
         <v>1</v>
       </c>
-      <c r="K27" s="32">
+      <c r="K27" s="28">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L27" s="75" t="s">
-        <v>191</v>
-      </c>
-      <c r="M27" s="33">
-        <v>0.29239999999999999</v>
-      </c>
-      <c r="N27" s="33">
+      <c r="L27" s="67" t="s">
+        <v>204</v>
+      </c>
+      <c r="M27" s="29">
+        <v>1.2</v>
+      </c>
+      <c r="N27" s="29">
         <f t="shared" si="1"/>
-        <v>0.29239999999999999</v>
-      </c>
-      <c r="O27" s="33">
-        <v>0.29239999999999999</v>
-      </c>
-      <c r="P27" s="33">
+        <v>1.2</v>
+      </c>
+      <c r="O27" s="29">
+        <v>1.2</v>
+      </c>
+      <c r="P27" s="29">
         <f t="shared" si="2"/>
-        <v>1.462</v>
-      </c>
-      <c r="Q27" s="34"/>
+        <v>6</v>
+      </c>
+      <c r="Q27" s="30"/>
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
     </row>
@@ -3114,56 +3114,56 @@
       <c r="A28" s="13">
         <v>26</v>
       </c>
-      <c r="B28" s="35" t="s">
-        <v>141</v>
-      </c>
-      <c r="C28" s="84" t="s">
-        <v>192</v>
-      </c>
-      <c r="D28" s="65" t="s">
+      <c r="B28" s="83" t="s">
+        <v>140</v>
+      </c>
+      <c r="C28" s="76" t="s">
+        <v>190</v>
+      </c>
+      <c r="D28" s="57" t="s">
+        <v>134</v>
+      </c>
+      <c r="E28" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="F28" s="77" t="s">
         <v>135</v>
       </c>
-      <c r="E28" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="F28" s="85" t="s">
-        <v>136</v>
-      </c>
-      <c r="G28" s="23" t="s">
-        <v>190</v>
+      <c r="G28" s="19" t="s">
+        <v>189</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>204</v>
-      </c>
-      <c r="I28" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="J28" s="45">
+        <v>202</v>
+      </c>
+      <c r="I28" s="20" t="s">
+        <v>138</v>
+      </c>
+      <c r="J28" s="38">
         <v>1</v>
       </c>
-      <c r="K28" s="25">
+      <c r="K28" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L28" s="26" t="s">
+      <c r="L28" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="M28" s="27">
+      <c r="M28" s="23">
         <v>0.84</v>
       </c>
-      <c r="N28" s="27">
+      <c r="N28" s="23">
         <f t="shared" si="1"/>
         <v>0.84</v>
       </c>
-      <c r="O28" s="27">
+      <c r="O28" s="23">
         <v>0.84</v>
       </c>
-      <c r="P28" s="27">
+      <c r="P28" s="23">
         <f t="shared" si="2"/>
         <v>4.2</v>
       </c>
-      <c r="Q28" s="86" t="s">
-        <v>205</v>
+      <c r="Q28" s="78" t="s">
+        <v>203</v>
       </c>
       <c r="R28" s="2"/>
       <c r="S28" s="2"/>
@@ -3172,53 +3172,53 @@
       <c r="A29" s="13">
         <v>27</v>
       </c>
-      <c r="B29" s="37"/>
-      <c r="C29" s="87" t="s">
-        <v>193</v>
-      </c>
-      <c r="D29" s="90" t="s">
+      <c r="B29" s="85"/>
+      <c r="C29" s="79" t="s">
+        <v>191</v>
+      </c>
+      <c r="D29" s="82" t="s">
+        <v>136</v>
+      </c>
+      <c r="E29" s="82" t="s">
+        <v>31</v>
+      </c>
+      <c r="F29" s="82" t="s">
         <v>137</v>
       </c>
-      <c r="E29" s="90" t="s">
-        <v>31</v>
-      </c>
-      <c r="F29" s="90" t="s">
-        <v>138</v>
-      </c>
-      <c r="G29" s="89" t="s">
-        <v>194</v>
-      </c>
-      <c r="H29" s="89" t="s">
-        <v>128</v>
-      </c>
-      <c r="I29" s="89" t="s">
-        <v>163</v>
-      </c>
-      <c r="J29" s="46">
+      <c r="G29" s="81" t="s">
+        <v>192</v>
+      </c>
+      <c r="H29" s="81" t="s">
+        <v>127</v>
+      </c>
+      <c r="I29" s="81" t="s">
+        <v>162</v>
+      </c>
+      <c r="J29" s="39">
         <v>1</v>
       </c>
-      <c r="K29" s="32">
+      <c r="K29" s="28">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L29" s="75" t="s">
-        <v>191</v>
-      </c>
-      <c r="M29" s="33">
-        <v>0.4148</v>
-      </c>
-      <c r="N29" s="33">
+      <c r="L29" s="67" t="s">
+        <v>204</v>
+      </c>
+      <c r="M29" s="29">
+        <v>1.6</v>
+      </c>
+      <c r="N29" s="29">
         <f t="shared" si="1"/>
-        <v>0.4148</v>
-      </c>
-      <c r="O29" s="33">
-        <v>0.4148</v>
-      </c>
-      <c r="P29" s="33">
+        <v>1.6</v>
+      </c>
+      <c r="O29" s="29">
+        <v>1.6</v>
+      </c>
+      <c r="P29" s="29">
         <f t="shared" si="2"/>
-        <v>2.0739999999999998</v>
-      </c>
-      <c r="Q29" s="34"/>
+        <v>8</v>
+      </c>
+      <c r="Q29" s="30"/>
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
     </row>
@@ -3226,55 +3226,55 @@
       <c r="A30" s="13">
         <v>28</v>
       </c>
-      <c r="B30" s="35" t="s">
+      <c r="B30" s="83" t="s">
         <v>28</v>
       </c>
-      <c r="C30" s="64" t="s">
+      <c r="C30" s="56" t="s">
+        <v>141</v>
+      </c>
+      <c r="D30" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="E30" s="31" t="s">
         <v>142</v>
       </c>
-      <c r="D30" s="38" t="s">
-        <v>42</v>
-      </c>
-      <c r="E30" s="38" t="s">
+      <c r="F30" s="31" t="s">
         <v>143</v>
       </c>
-      <c r="F30" s="38" t="s">
-        <v>144</v>
-      </c>
-      <c r="G30" s="23" t="s">
-        <v>179</v>
-      </c>
-      <c r="H30" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="I30" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="J30" s="45">
+      <c r="G30" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="H30" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="I30" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="J30" s="38">
         <v>1</v>
       </c>
-      <c r="K30" s="25">
+      <c r="K30" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L30" s="66" t="s">
+      <c r="L30" s="58" t="s">
         <v>30</v>
       </c>
-      <c r="M30" s="27">
+      <c r="M30" s="23">
         <v>5.8</v>
       </c>
-      <c r="N30" s="27">
+      <c r="N30" s="23">
         <f t="shared" si="1"/>
         <v>5.8</v>
       </c>
-      <c r="O30" s="27">
+      <c r="O30" s="23">
         <v>5.8</v>
       </c>
-      <c r="P30" s="27">
+      <c r="P30" s="23">
         <f t="shared" si="2"/>
         <v>29</v>
       </c>
-      <c r="Q30" s="28"/>
+      <c r="Q30" s="24"/>
       <c r="R30" s="2"/>
       <c r="S30" s="2"/>
     </row>
@@ -3282,27 +3282,27 @@
       <c r="A31" s="13">
         <v>29</v>
       </c>
-      <c r="B31" s="36"/>
-      <c r="C31" s="67" t="s">
-        <v>145</v>
+      <c r="B31" s="84"/>
+      <c r="C31" s="59" t="s">
+        <v>144</v>
       </c>
       <c r="D31" s="14" t="s">
         <v>43</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J31" s="12">
         <v>1</v>
@@ -3328,7 +3328,7 @@
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="Q31" s="29"/>
+      <c r="Q31" s="25"/>
       <c r="R31" s="2"/>
       <c r="S31" s="2"/>
     </row>
@@ -3336,27 +3336,27 @@
       <c r="A32" s="13">
         <v>30</v>
       </c>
-      <c r="B32" s="36"/>
-      <c r="C32" s="67" t="s">
-        <v>147</v>
+      <c r="B32" s="84"/>
+      <c r="C32" s="59" t="s">
+        <v>146</v>
       </c>
       <c r="D32" s="14" t="s">
         <v>44</v>
       </c>
       <c r="E32" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="F32" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="F32" s="14" t="s">
-        <v>149</v>
-      </c>
       <c r="G32" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J32" s="12">
         <v>1</v>
@@ -3366,7 +3366,7 @@
         <v>5</v>
       </c>
       <c r="L32" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="M32" s="6">
         <v>0.45</v>
@@ -3382,7 +3382,7 @@
         <f t="shared" si="2"/>
         <v>2.25</v>
       </c>
-      <c r="Q32" s="29"/>
+      <c r="Q32" s="25"/>
       <c r="R32" s="2"/>
       <c r="S32" s="2"/>
     </row>
@@ -3390,27 +3390,27 @@
       <c r="A33" s="13">
         <v>31</v>
       </c>
-      <c r="B33" s="36"/>
-      <c r="C33" s="70" t="s">
-        <v>184</v>
+      <c r="B33" s="84"/>
+      <c r="C33" s="62" t="s">
+        <v>183</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>31</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J33" s="12">
         <v>4</v>
@@ -3420,7 +3420,7 @@
         <v>20</v>
       </c>
       <c r="L33" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="M33" s="6">
         <v>0.81</v>
@@ -3436,7 +3436,7 @@
         <f t="shared" si="2"/>
         <v>16.200000000000003</v>
       </c>
-      <c r="Q33" s="29"/>
+      <c r="Q33" s="25"/>
       <c r="R33" s="2"/>
       <c r="S33" s="2"/>
     </row>
@@ -3444,27 +3444,27 @@
       <c r="A34" s="13">
         <v>32</v>
       </c>
-      <c r="B34" s="36"/>
-      <c r="C34" s="67" t="s">
-        <v>152</v>
+      <c r="B34" s="84"/>
+      <c r="C34" s="59" t="s">
+        <v>151</v>
       </c>
       <c r="D34" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E34" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="F34" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="F34" s="14" t="s">
-        <v>154</v>
-      </c>
       <c r="G34" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J34" s="12">
         <v>1</v>
@@ -3490,7 +3490,7 @@
         <f t="shared" si="2"/>
         <v>6.3</v>
       </c>
-      <c r="Q34" s="29"/>
+      <c r="Q34" s="25"/>
       <c r="R34" s="2"/>
       <c r="S34" s="2"/>
     </row>
@@ -3498,53 +3498,53 @@
       <c r="A35" s="13">
         <v>33</v>
       </c>
-      <c r="B35" s="37"/>
-      <c r="C35" s="76" t="s">
+      <c r="B35" s="85"/>
+      <c r="C35" s="68" t="s">
+        <v>184</v>
+      </c>
+      <c r="D35" s="66" t="s">
+        <v>154</v>
+      </c>
+      <c r="E35" s="27" t="s">
         <v>185</v>
       </c>
-      <c r="D35" s="74" t="s">
+      <c r="F35" s="66" t="s">
         <v>155</v>
       </c>
-      <c r="E35" s="31" t="s">
+      <c r="G35" s="26" t="s">
         <v>186</v>
       </c>
-      <c r="F35" s="74" t="s">
-        <v>156</v>
-      </c>
-      <c r="G35" s="30" t="s">
-        <v>187</v>
-      </c>
-      <c r="H35" s="30" t="s">
-        <v>128</v>
-      </c>
-      <c r="I35" s="30" t="s">
-        <v>128</v>
-      </c>
-      <c r="J35" s="46">
+      <c r="H35" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="I35" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="J35" s="39">
         <v>5</v>
       </c>
-      <c r="K35" s="32">
+      <c r="K35" s="28">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="L35" s="75" t="s">
+      <c r="L35" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="M35" s="33">
+      <c r="M35" s="29">
         <v>0.48</v>
       </c>
-      <c r="N35" s="33">
+      <c r="N35" s="29">
         <f t="shared" si="1"/>
         <v>2.4</v>
       </c>
-      <c r="O35" s="33">
+      <c r="O35" s="29">
         <v>0.48</v>
       </c>
-      <c r="P35" s="33">
+      <c r="P35" s="29">
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="Q35" s="34"/>
+      <c r="Q35" s="30"/>
       <c r="R35" s="2"/>
       <c r="S35" s="2"/>
     </row>
@@ -3552,55 +3552,55 @@
       <c r="A36" s="13">
         <v>34</v>
       </c>
-      <c r="B36" s="35" t="s">
+      <c r="B36" s="83" t="s">
         <v>29</v>
       </c>
-      <c r="C36" s="64" t="s">
+      <c r="C36" s="56" t="s">
         <v>48</v>
       </c>
-      <c r="D36" s="38" t="s">
+      <c r="D36" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E36" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="F36" s="31" t="s">
         <v>157</v>
       </c>
-      <c r="E36" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="F36" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="G36" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="H36" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="I36" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="J36" s="45">
+      <c r="G36" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="H36" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="I36" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="J36" s="38">
         <v>5</v>
       </c>
-      <c r="K36" s="25">
+      <c r="K36" s="21">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="L36" s="66" t="s">
-        <v>188</v>
-      </c>
-      <c r="M36" s="27">
+      <c r="L36" s="58" t="s">
+        <v>187</v>
+      </c>
+      <c r="M36" s="23">
         <v>0.17347000000000001</v>
       </c>
-      <c r="N36" s="27">
+      <c r="N36" s="23">
         <f t="shared" si="1"/>
         <v>0.86735000000000007</v>
       </c>
-      <c r="O36" s="27">
+      <c r="O36" s="23">
         <v>0.17347000000000001</v>
       </c>
-      <c r="P36" s="27">
+      <c r="P36" s="23">
         <f t="shared" si="2"/>
         <v>4.3367500000000003</v>
       </c>
-      <c r="Q36" s="28"/>
+      <c r="Q36" s="24"/>
       <c r="R36" s="2"/>
       <c r="S36" s="2"/>
     </row>
@@ -3608,27 +3608,27 @@
       <c r="A37" s="13">
         <v>35</v>
       </c>
-      <c r="B37" s="36"/>
-      <c r="C37" s="70" t="s">
-        <v>202</v>
+      <c r="B37" s="84"/>
+      <c r="C37" s="62" t="s">
+        <v>200</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E37" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="F37" s="69" t="s">
-        <v>160</v>
+      <c r="F37" s="61" t="s">
+        <v>159</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H37" s="3">
         <v>1715857</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J37" s="12">
         <v>2</v>
@@ -3654,7 +3654,7 @@
         <f t="shared" si="2"/>
         <v>21.9</v>
       </c>
-      <c r="Q37" s="29"/>
+      <c r="Q37" s="25"/>
       <c r="R37" s="2"/>
       <c r="S37" s="2"/>
     </row>
@@ -3662,8 +3662,8 @@
       <c r="A38" s="13">
         <v>36</v>
       </c>
-      <c r="B38" s="36"/>
-      <c r="C38" s="67" t="s">
+      <c r="B38" s="84"/>
+      <c r="C38" s="59" t="s">
         <v>9</v>
       </c>
       <c r="D38" s="14" t="s">
@@ -3676,13 +3676,13 @@
         <v>8</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J38" s="12">
         <v>1</v>
@@ -3708,93 +3708,93 @@
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="Q38" s="29"/>
+      <c r="Q38" s="25"/>
       <c r="R38" s="2"/>
       <c r="S38" s="2"/>
     </row>
     <row r="39" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="63">
+      <c r="A39" s="55">
         <v>37</v>
       </c>
-      <c r="B39" s="37"/>
-      <c r="C39" s="72" t="s">
+      <c r="B39" s="85"/>
+      <c r="C39" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="D39" s="74" t="s">
+      <c r="D39" s="66" t="s">
+        <v>160</v>
+      </c>
+      <c r="E39" s="66" t="s">
+        <v>31</v>
+      </c>
+      <c r="F39" s="66" t="s">
         <v>161</v>
       </c>
-      <c r="E39" s="74" t="s">
-        <v>31</v>
-      </c>
-      <c r="F39" s="74" t="s">
-        <v>162</v>
-      </c>
-      <c r="G39" s="30" t="s">
-        <v>189</v>
-      </c>
-      <c r="H39" s="30" t="s">
-        <v>128</v>
-      </c>
-      <c r="I39" s="30" t="s">
-        <v>128</v>
-      </c>
-      <c r="J39" s="46">
+      <c r="G39" s="26" t="s">
+        <v>188</v>
+      </c>
+      <c r="H39" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="I39" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="J39" s="39">
         <v>1</v>
       </c>
-      <c r="K39" s="32">
+      <c r="K39" s="28">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L39" s="75" t="s">
+      <c r="L39" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="M39" s="33">
+      <c r="M39" s="29">
         <v>0.45</v>
       </c>
-      <c r="N39" s="33">
+      <c r="N39" s="29">
         <f t="shared" si="1"/>
         <v>0.45</v>
       </c>
-      <c r="O39" s="33">
+      <c r="O39" s="29">
         <v>0.45</v>
       </c>
-      <c r="P39" s="33">
+      <c r="P39" s="29">
         <f t="shared" si="2"/>
         <v>2.25</v>
       </c>
-      <c r="Q39" s="61"/>
+      <c r="Q39" s="53"/>
       <c r="R39" s="2"/>
       <c r="S39" s="2"/>
     </row>
     <row r="40" spans="1:19" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H40" s="60" t="s">
+      <c r="H40" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="I40" s="60"/>
-      <c r="J40" s="60"/>
+      <c r="I40" s="86"/>
+      <c r="J40" s="86"/>
       <c r="N40" s="17">
         <f>SUM(N3:N39)</f>
-        <v>41.894549999999995</v>
+        <v>43.987349999999999</v>
       </c>
       <c r="O40" s="7"/>
       <c r="P40" s="15">
         <f>SUM(P3:P39)</f>
-        <v>190.24875</v>
+        <v>200.71275</v>
       </c>
       <c r="R40" s="2"/>
       <c r="S40" s="2"/>
     </row>
     <row r="41" spans="1:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H41" s="19" t="s">
+      <c r="H41" s="87" t="s">
         <v>33</v>
       </c>
-      <c r="I41" s="19"/>
-      <c r="J41" s="19"/>
+      <c r="I41" s="87"/>
+      <c r="J41" s="87"/>
       <c r="N41" s="18"/>
       <c r="O41" s="8"/>
       <c r="P41" s="9">
         <f>P40/5</f>
-        <v>38.049750000000003</v>
+        <v>40.14255</v>
       </c>
       <c r="R41" s="2"/>
       <c r="S41" s="2"/>
@@ -4028,15 +4028,14 @@
     <hyperlink ref="L36" r:id="rId29"/>
     <hyperlink ref="L38" r:id="rId30"/>
     <hyperlink ref="L39" r:id="rId31"/>
-    <hyperlink ref="L27" r:id="rId32"/>
-    <hyperlink ref="L29" r:id="rId33"/>
-    <hyperlink ref="L21" r:id="rId34"/>
-    <hyperlink ref="L37" r:id="rId35"/>
-    <hyperlink ref="L8" r:id="rId36"/>
-    <hyperlink ref="L28" r:id="rId37"/>
+    <hyperlink ref="L29" r:id="rId32" display="LCSC"/>
+    <hyperlink ref="L21" r:id="rId33"/>
+    <hyperlink ref="L37" r:id="rId34"/>
+    <hyperlink ref="L8" r:id="rId35"/>
+    <hyperlink ref="L28" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId38"/>
+  <pageSetup orientation="portrait" r:id="rId37"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>